<commit_message>
Auto-cochage de la fonction du bungalow + durcissement Windows
- Fonction bungalow : détection bloc->fonction config-driven (app/fonctions.py +
  section `fonctions:` de cellules.yaml), report sur EtatDesLieux.fonction (assemblage),
  remplacement de la cellule fonction dans remplissage.py. Tests (test_fonctions.py).
- Durcissement Windows (console cp1252) : seed_demo, diagnostic, make_placeholder_templates
  et hash_password forcent la sortie en UTF-8 (corrige des plantages réels sur ✔/→).
- Docs : CLAUDE.md (état d'avancement, pièges Windows, déploiement disque local).

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/templates/bungalow_15m2.xlsx
+++ b/templates/bungalow_15m2.xlsx
@@ -596,6 +596,18 @@
       </c>
       <c r="E18" s="3" t="n"/>
     </row>
+    <row r="20">
+      <c r="A20" s="2" t="inlineStr">
+        <is>
+          <t>Fonction</t>
+        </is>
+      </c>
+      <c r="B20" s="3" t="inlineStr">
+        <is>
+          <t>BUREAU / SALLE DE REUNION / VESTIAIRE / REFECTOIRE</t>
+        </is>
+      </c>
+    </row>
     <row r="22">
       <c r="A22" s="4" t="inlineStr">
         <is>

</xml_diff>